<commit_message>
remove dominant detection in commits for simplicity
</commit_message>
<xml_diff>
--- a/results/tables/commitizen/compare/consolidated_results_table_anomaly_categories.xlsx
+++ b/results/tables/commitizen/compare/consolidated_results_table_anomaly_categories.xlsx
@@ -8,14 +8,27 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://campusfl-my.sharepoint.com/personal/mahsa_choopannezhad_uni_li/Documents/Desktop/PhD materials/codes/Lifecycles-Processes/results/tables/commitizen/compare/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="8_{FB6ABDC3-565B-4E76-AAEA-DF95D21D7E46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9096CACB-51AB-4115-8913-00049DE71D4A}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="8_{FB6ABDC3-565B-4E76-AAEA-DF95D21D7E46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{87F1C897-F1EA-4DFF-85E0-A160B1D75A64}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D91BF3F4-C40A-4697-BB76-36024B251428}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{D91BF3F4-C40A-4697-BB76-36024B251428}"/>
   </bookViews>
   <sheets>
     <sheet name="consolidated_results_table_anom" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -655,6 +668,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1486,8 +1503,8 @@
         <v>0.55828572787792852</v>
       </c>
       <c r="O12" s="1">
-        <f>AVERAGE(I2:I7)</f>
-        <v>0.5708139378489907</v>
+        <f>AVERAGE(I2:I6)</f>
+        <v>0.55811914285958542</v>
       </c>
       <c r="P12" s="1">
         <f>(C2*I2+C3*I3+C4*I4+C5*I5+C6*I6+C7*I7+C8*I8+C9*I9+C10*I10+C11*I11)/C12</f>
@@ -1958,8 +1975,8 @@
         <v>0.43088911762782239</v>
       </c>
       <c r="O23">
-        <f>AVERAGE(I13:I18)</f>
-        <v>0.41170183522950815</v>
+        <f>AVERAGE(I13:I17)</f>
+        <v>0.39255478503285884</v>
       </c>
       <c r="P23" s="1">
         <f>(C13*I13+C14*I14+C15*I15+C16*I16+C17*I17+C18*I18+C19*I19+C20*I20+C21*I21+C22*I22)/C23</f>
@@ -2430,8 +2447,8 @@
         <v>0.65703573826940675</v>
       </c>
       <c r="O34" s="1">
-        <f>AVERAGE(I24:I29)</f>
-        <v>0.67583008571486891</v>
+        <f>AVERAGE(I24:I28)</f>
+        <v>0.70307632042001744</v>
       </c>
       <c r="P34" s="1">
         <f>(C24*I24+C25*I25+C26*I26+C27*I27+C28*I28+C29*I29+C30*I30+C31*I31+C32*I32+C33*I33)/C34</f>

</xml_diff>